<commit_message>
Updated chart title for results
</commit_message>
<xml_diff>
--- a/result_analysis.xlsx
+++ b/result_analysis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tintin/Desktop/Projects/credit_risk_model/result_analysis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tintin/Desktop/Projects/credit_risk_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B792EA5-9AF6-E945-B565-DA255D487101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69FA589-4733-0A40-BB06-0C058002A156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="800" windowWidth="28040" windowHeight="17440" activeTab="3" xr2:uid="{61FC1A9A-6CB0-D841-9DA7-4D6ECF9C438C}"/>
+    <workbookView xWindow="1100" yWindow="780" windowWidth="28040" windowHeight="17440" activeTab="3" xr2:uid="{61FC1A9A-6CB0-D841-9DA7-4D6ECF9C438C}"/>
   </bookViews>
   <sheets>
     <sheet name="raw_data" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="33" r:id="rId5"/>
+    <pivotCache cacheId="34" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -167,7 +167,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -238,7 +238,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -246,24 +246,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="175" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="10" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="175" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -271,18 +270,37 @@
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="7" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -301,7 +319,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="175" formatCode="&quot;$&quot;#,##0"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
     </dxf>
     <dxf>
       <font>
@@ -342,37 +360,18 @@
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="7" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -427,11 +426,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Maximize</a:t>
+              <a:t>Maximum</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Profit against Predicted Probability of Default</a:t>
+              <a:t> Profit from Model Predicted Default Probability</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -5570,7 +5569,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2363CDFC-DF88-C74D-8AF0-219FA876DE04}" name="PivotTable1" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Decile">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2363CDFC-DF88-C74D-8AF0-219FA876DE04}" name="PivotTable1" cacheId="34" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Decile">
   <location ref="A3:D14" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField showAll="0"/>
@@ -5653,7 +5652,7 @@
     <dataField name="Min of Probability_Default" fld="3" subtotal="min" baseField="0" baseItem="0" numFmtId="10"/>
   </dataFields>
   <formats count="2">
-    <format dxfId="1">
+    <format dxfId="10">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5665,7 +5664,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="0">
+    <format dxfId="9">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="2">
           <reference field="4294967294" count="1" selected="0">
@@ -5695,7 +5694,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}" name="Table1" displayName="Table1" ref="A1:G401" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}" name="Table1" displayName="Table1" ref="A1:G401" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:G401" xr:uid="{00A61614-C026-F049-8D7D-B2C5D987FC7D}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E401">
     <sortCondition descending="1" ref="D1:D401"/>
@@ -5703,13 +5702,13 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{A33D2E8F-C4FE-744C-B6EA-6D08D082939C}" name="index"/>
     <tableColumn id="2" xr3:uid="{B6ED8025-A452-0545-83F5-078527E9E23D}" name="Actual Outcome"/>
-    <tableColumn id="3" xr3:uid="{482B43F2-766E-4344-A44D-179FE0BFAA6E}" name="Probability_Safe" dataDxfId="9" dataCellStyle="Percent"/>
-    <tableColumn id="4" xr3:uid="{797E6CBE-CC91-DD44-BA30-CDAD50AEEDE6}" name="Probability_Default" dataDxfId="8" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{482B43F2-766E-4344-A44D-179FE0BFAA6E}" name="Probability_Safe" dataDxfId="4" dataCellStyle="Percent"/>
+    <tableColumn id="4" xr3:uid="{797E6CBE-CC91-DD44-BA30-CDAD50AEEDE6}" name="Probability_Default" dataDxfId="3" dataCellStyle="Percent"/>
     <tableColumn id="5" xr3:uid="{8F649A08-FC6F-404F-ADA2-2B66671FF421}" name="Predicted Outcome"/>
-    <tableColumn id="8" xr3:uid="{B81D5698-9F0B-9B45-A8E1-F4463C47F39B}" name="True Positive" dataDxfId="5">
+    <tableColumn id="8" xr3:uid="{B81D5698-9F0B-9B45-A8E1-F4463C47F39B}" name="True Positive" dataDxfId="2">
       <calculatedColumnFormula>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{47E82062-EA15-D14E-9771-A0661A0DD882}" name="Decile" dataDxfId="6">
+    <tableColumn id="7" xr3:uid="{47E82062-EA15-D14E-9771-A0661A0DD882}" name="Decile" dataDxfId="1">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(MAX(IF(Table2[Probability_Default]&lt;Table1[[#This Row],[Probability_Default]],Table2[Probability_Default])),Table2[Probability_Default],Table2[Decile],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5722,7 +5721,7 @@
   <autoFilter ref="J1:K10" xr:uid="{67FE4D2D-295A-FD43-B1A1-4828D3A56142}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{85908CF2-458E-DC4E-9C8D-DD7ACB04BE26}" name="Decile"/>
-    <tableColumn id="2" xr3:uid="{829CD0D6-0304-6044-B4C2-6E080E4914FE}" name="Probability_Default" dataDxfId="7" dataCellStyle="Percent"/>
+    <tableColumn id="2" xr3:uid="{829CD0D6-0304-6044-B4C2-6E080E4914FE}" name="Probability_Default" dataDxfId="0" dataCellStyle="Percent"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5753,16 +5752,16 @@
     <tableColumn id="3" xr3:uid="{4DF9A59C-7522-3B4F-9E93-B8FD4567A10D}" name="Cumulative Defaults">
       <calculatedColumnFormula>SUM($C$4:C4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{0B23C047-C32D-3A4B-BD60-B8C615AA7BB4}" name="Cumulative % of Defaults" dataDxfId="4" dataCellStyle="Percent">
+    <tableColumn id="5" xr3:uid="{0B23C047-C32D-3A4B-BD60-B8C615AA7BB4}" name="Cumulative % of Defaults" dataDxfId="8" dataCellStyle="Percent">
       <calculatedColumnFormula>(H4)/$H$13</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{F7D20E3F-556C-1940-82F2-43B673E2D5D4}" name="Cumulative Safe Loans">
       <calculatedColumnFormula>SUM($G$4:G4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{828E05FA-42DB-2D44-82BC-3CE97F0BCB66}" name="Cumulative % of Safe Loans" dataDxfId="3" dataCellStyle="Percent">
+    <tableColumn id="6" xr3:uid="{828E05FA-42DB-2D44-82BC-3CE97F0BCB66}" name="Cumulative % of Safe Loans" dataDxfId="7" dataCellStyle="Percent">
       <calculatedColumnFormula>(J4)/$J$13</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B38B3630-1B13-C646-85B9-356D48FF1C8B}" name="Total Profit" dataDxfId="2" dataCellStyle="Percent">
+    <tableColumn id="4" xr3:uid="{B38B3630-1B13-C646-85B9-356D48FF1C8B}" name="Total Profit" dataDxfId="6" dataCellStyle="Percent">
       <calculatedColumnFormula>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -13307,7 +13306,7 @@
     <col min="2" max="2" width="17.6640625" customWidth="1"/>
     <col min="3" max="4" width="20.5" style="2" customWidth="1"/>
     <col min="5" max="5" width="22.33203125" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="7" customWidth="1"/>
     <col min="7" max="7" width="21.33203125" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="20.1640625" customWidth="1"/>
@@ -13329,7 +13328,7 @@
       <c r="E1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>19</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -13358,7 +13357,7 @@
       <c r="E2">
         <v>1</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13390,7 +13389,7 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13422,7 +13421,7 @@
       <c r="E4">
         <v>1</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13454,7 +13453,7 @@
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13486,7 +13485,7 @@
       <c r="E6">
         <v>1</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13518,7 +13517,7 @@
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13550,7 +13549,7 @@
       <c r="E8">
         <v>1</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13582,7 +13581,7 @@
       <c r="E9">
         <v>1</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13614,7 +13613,7 @@
       <c r="E10">
         <v>1</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -13646,7 +13645,7 @@
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -13671,7 +13670,7 @@
       <c r="E12">
         <v>1</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13696,7 +13695,7 @@
       <c r="E13">
         <v>1</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -13721,7 +13720,7 @@
       <c r="E14">
         <v>1</v>
       </c>
-      <c r="F14" s="8">
+      <c r="F14" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13746,7 +13745,7 @@
       <c r="E15">
         <v>1</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13771,7 +13770,7 @@
       <c r="E16">
         <v>1</v>
       </c>
-      <c r="F16" s="8">
+      <c r="F16" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13796,7 +13795,7 @@
       <c r="E17">
         <v>1</v>
       </c>
-      <c r="F17" s="8">
+      <c r="F17" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13821,7 +13820,7 @@
       <c r="E18">
         <v>1</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -13846,7 +13845,7 @@
       <c r="E19">
         <v>1</v>
       </c>
-      <c r="F19" s="8">
+      <c r="F19" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13871,7 +13870,7 @@
       <c r="E20">
         <v>1</v>
       </c>
-      <c r="F20" s="8">
+      <c r="F20" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13896,7 +13895,7 @@
       <c r="E21">
         <v>1</v>
       </c>
-      <c r="F21" s="8">
+      <c r="F21" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -13921,7 +13920,7 @@
       <c r="E22">
         <v>1</v>
       </c>
-      <c r="F22" s="8">
+      <c r="F22" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13946,7 +13945,7 @@
       <c r="E23">
         <v>1</v>
       </c>
-      <c r="F23" s="8">
+      <c r="F23" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13971,7 +13970,7 @@
       <c r="E24">
         <v>1</v>
       </c>
-      <c r="F24" s="8">
+      <c r="F24" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -13996,7 +13995,7 @@
       <c r="E25">
         <v>1</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14021,7 +14020,7 @@
       <c r="E26">
         <v>1</v>
       </c>
-      <c r="F26" s="8">
+      <c r="F26" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14050,7 +14049,7 @@
       <c r="E27">
         <v>1</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14079,7 +14078,7 @@
       <c r="E28">
         <v>1</v>
       </c>
-      <c r="F28" s="8">
+      <c r="F28" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14104,7 +14103,7 @@
       <c r="E29">
         <v>1</v>
       </c>
-      <c r="F29" s="8">
+      <c r="F29" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14129,7 +14128,7 @@
       <c r="E30">
         <v>1</v>
       </c>
-      <c r="F30" s="8">
+      <c r="F30" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14154,7 +14153,7 @@
       <c r="E31">
         <v>1</v>
       </c>
-      <c r="F31" s="8">
+      <c r="F31" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14179,7 +14178,7 @@
       <c r="E32">
         <v>1</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14204,7 +14203,7 @@
       <c r="E33">
         <v>1</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14229,7 +14228,7 @@
       <c r="E34">
         <v>1</v>
       </c>
-      <c r="F34" s="8">
+      <c r="F34" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14254,7 +14253,7 @@
       <c r="E35">
         <v>1</v>
       </c>
-      <c r="F35" s="8">
+      <c r="F35" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14279,7 +14278,7 @@
       <c r="E36">
         <v>1</v>
       </c>
-      <c r="F36" s="8">
+      <c r="F36" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14304,7 +14303,7 @@
       <c r="E37">
         <v>1</v>
       </c>
-      <c r="F37" s="8">
+      <c r="F37" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14329,7 +14328,7 @@
       <c r="E38">
         <v>1</v>
       </c>
-      <c r="F38" s="8">
+      <c r="F38" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14354,7 +14353,7 @@
       <c r="E39">
         <v>1</v>
       </c>
-      <c r="F39" s="8">
+      <c r="F39" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14379,7 +14378,7 @@
       <c r="E40">
         <v>1</v>
       </c>
-      <c r="F40" s="8">
+      <c r="F40" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14404,7 +14403,7 @@
       <c r="E41">
         <v>1</v>
       </c>
-      <c r="F41" s="8">
+      <c r="F41" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14429,7 +14428,7 @@
       <c r="E42">
         <v>1</v>
       </c>
-      <c r="F42" s="8">
+      <c r="F42" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14454,7 +14453,7 @@
       <c r="E43">
         <v>1</v>
       </c>
-      <c r="F43" s="8">
+      <c r="F43" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14479,7 +14478,7 @@
       <c r="E44">
         <v>1</v>
       </c>
-      <c r="F44" s="8">
+      <c r="F44" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14504,7 +14503,7 @@
       <c r="E45">
         <v>1</v>
       </c>
-      <c r="F45" s="8">
+      <c r="F45" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14529,7 +14528,7 @@
       <c r="E46">
         <v>1</v>
       </c>
-      <c r="F46" s="8">
+      <c r="F46" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14554,7 +14553,7 @@
       <c r="E47">
         <v>1</v>
       </c>
-      <c r="F47" s="8">
+      <c r="F47" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14579,7 +14578,7 @@
       <c r="E48">
         <v>1</v>
       </c>
-      <c r="F48" s="8">
+      <c r="F48" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14604,7 +14603,7 @@
       <c r="E49">
         <v>1</v>
       </c>
-      <c r="F49" s="8">
+      <c r="F49" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14629,7 +14628,7 @@
       <c r="E50">
         <v>1</v>
       </c>
-      <c r="F50" s="8">
+      <c r="F50" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14654,7 +14653,7 @@
       <c r="E51">
         <v>1</v>
       </c>
-      <c r="F51" s="8">
+      <c r="F51" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14679,7 +14678,7 @@
       <c r="E52">
         <v>1</v>
       </c>
-      <c r="F52" s="8">
+      <c r="F52" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14704,7 +14703,7 @@
       <c r="E53">
         <v>1</v>
       </c>
-      <c r="F53" s="8">
+      <c r="F53" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14729,7 +14728,7 @@
       <c r="E54">
         <v>1</v>
       </c>
-      <c r="F54" s="8">
+      <c r="F54" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -14754,7 +14753,7 @@
       <c r="E55">
         <v>1</v>
       </c>
-      <c r="F55" s="8">
+      <c r="F55" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14779,7 +14778,7 @@
       <c r="E56">
         <v>1</v>
       </c>
-      <c r="F56" s="8">
+      <c r="F56" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14804,7 +14803,7 @@
       <c r="E57">
         <v>1</v>
       </c>
-      <c r="F57" s="8">
+      <c r="F57" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14829,7 +14828,7 @@
       <c r="E58">
         <v>1</v>
       </c>
-      <c r="F58" s="8">
+      <c r="F58" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14854,7 +14853,7 @@
       <c r="E59">
         <v>1</v>
       </c>
-      <c r="F59" s="8">
+      <c r="F59" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14879,7 +14878,7 @@
       <c r="E60">
         <v>1</v>
       </c>
-      <c r="F60" s="8">
+      <c r="F60" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14904,7 +14903,7 @@
       <c r="E61">
         <v>1</v>
       </c>
-      <c r="F61" s="8">
+      <c r="F61" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14929,7 +14928,7 @@
       <c r="E62">
         <v>1</v>
       </c>
-      <c r="F62" s="8">
+      <c r="F62" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14954,7 +14953,7 @@
       <c r="E63">
         <v>1</v>
       </c>
-      <c r="F63" s="8">
+      <c r="F63" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -14979,7 +14978,7 @@
       <c r="E64">
         <v>1</v>
       </c>
-      <c r="F64" s="8">
+      <c r="F64" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15004,7 +15003,7 @@
       <c r="E65">
         <v>1</v>
       </c>
-      <c r="F65" s="8">
+      <c r="F65" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15029,7 +15028,7 @@
       <c r="E66">
         <v>1</v>
       </c>
-      <c r="F66" s="8">
+      <c r="F66" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15054,7 +15053,7 @@
       <c r="E67">
         <v>1</v>
       </c>
-      <c r="F67" s="8">
+      <c r="F67" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15079,7 +15078,7 @@
       <c r="E68">
         <v>1</v>
       </c>
-      <c r="F68" s="8">
+      <c r="F68" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15104,7 +15103,7 @@
       <c r="E69">
         <v>1</v>
       </c>
-      <c r="F69" s="8">
+      <c r="F69" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15129,7 +15128,7 @@
       <c r="E70">
         <v>1</v>
       </c>
-      <c r="F70" s="8">
+      <c r="F70" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15154,7 +15153,7 @@
       <c r="E71">
         <v>1</v>
       </c>
-      <c r="F71" s="8">
+      <c r="F71" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15179,7 +15178,7 @@
       <c r="E72">
         <v>1</v>
       </c>
-      <c r="F72" s="8">
+      <c r="F72" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15204,7 +15203,7 @@
       <c r="E73">
         <v>1</v>
       </c>
-      <c r="F73" s="8">
+      <c r="F73" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15229,7 +15228,7 @@
       <c r="E74">
         <v>1</v>
       </c>
-      <c r="F74" s="8">
+      <c r="F74" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15254,7 +15253,7 @@
       <c r="E75">
         <v>1</v>
       </c>
-      <c r="F75" s="8">
+      <c r="F75" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15279,7 +15278,7 @@
       <c r="E76">
         <v>1</v>
       </c>
-      <c r="F76" s="8">
+      <c r="F76" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15304,7 +15303,7 @@
       <c r="E77">
         <v>1</v>
       </c>
-      <c r="F77" s="8">
+      <c r="F77" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15329,7 +15328,7 @@
       <c r="E78">
         <v>1</v>
       </c>
-      <c r="F78" s="8">
+      <c r="F78" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15354,7 +15353,7 @@
       <c r="E79">
         <v>1</v>
       </c>
-      <c r="F79" s="8">
+      <c r="F79" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15379,7 +15378,7 @@
       <c r="E80">
         <v>1</v>
       </c>
-      <c r="F80" s="8">
+      <c r="F80" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15404,7 +15403,7 @@
       <c r="E81">
         <v>1</v>
       </c>
-      <c r="F81" s="8">
+      <c r="F81" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15429,7 +15428,7 @@
       <c r="E82">
         <v>1</v>
       </c>
-      <c r="F82" s="8">
+      <c r="F82" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15454,7 +15453,7 @@
       <c r="E83">
         <v>1</v>
       </c>
-      <c r="F83" s="8">
+      <c r="F83" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15479,7 +15478,7 @@
       <c r="E84">
         <v>1</v>
       </c>
-      <c r="F84" s="8">
+      <c r="F84" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15504,7 +15503,7 @@
       <c r="E85">
         <v>1</v>
       </c>
-      <c r="F85" s="8">
+      <c r="F85" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15529,7 +15528,7 @@
       <c r="E86">
         <v>1</v>
       </c>
-      <c r="F86" s="8">
+      <c r="F86" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15554,7 +15553,7 @@
       <c r="E87">
         <v>1</v>
       </c>
-      <c r="F87" s="8">
+      <c r="F87" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15579,7 +15578,7 @@
       <c r="E88">
         <v>1</v>
       </c>
-      <c r="F88" s="8">
+      <c r="F88" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15604,7 +15603,7 @@
       <c r="E89">
         <v>1</v>
       </c>
-      <c r="F89" s="8">
+      <c r="F89" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15629,7 +15628,7 @@
       <c r="E90">
         <v>1</v>
       </c>
-      <c r="F90" s="8">
+      <c r="F90" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15654,7 +15653,7 @@
       <c r="E91">
         <v>1</v>
       </c>
-      <c r="F91" s="8">
+      <c r="F91" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15679,7 +15678,7 @@
       <c r="E92">
         <v>1</v>
       </c>
-      <c r="F92" s="8">
+      <c r="F92" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15704,7 +15703,7 @@
       <c r="E93">
         <v>1</v>
       </c>
-      <c r="F93" s="8">
+      <c r="F93" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15729,7 +15728,7 @@
       <c r="E94">
         <v>1</v>
       </c>
-      <c r="F94" s="8">
+      <c r="F94" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15754,7 +15753,7 @@
       <c r="E95">
         <v>1</v>
       </c>
-      <c r="F95" s="8">
+      <c r="F95" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15779,7 +15778,7 @@
       <c r="E96">
         <v>1</v>
       </c>
-      <c r="F96" s="8">
+      <c r="F96" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15804,7 +15803,7 @@
       <c r="E97">
         <v>1</v>
       </c>
-      <c r="F97" s="8">
+      <c r="F97" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15829,7 +15828,7 @@
       <c r="E98">
         <v>1</v>
       </c>
-      <c r="F98" s="8">
+      <c r="F98" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15854,7 +15853,7 @@
       <c r="E99">
         <v>1</v>
       </c>
-      <c r="F99" s="8">
+      <c r="F99" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15879,7 +15878,7 @@
       <c r="E100">
         <v>1</v>
       </c>
-      <c r="F100" s="8">
+      <c r="F100" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15904,7 +15903,7 @@
       <c r="E101">
         <v>1</v>
       </c>
-      <c r="F101" s="8">
+      <c r="F101" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15929,7 +15928,7 @@
       <c r="E102">
         <v>1</v>
       </c>
-      <c r="F102" s="8">
+      <c r="F102" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -15954,7 +15953,7 @@
       <c r="E103">
         <v>1</v>
       </c>
-      <c r="F103" s="8">
+      <c r="F103" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -15979,7 +15978,7 @@
       <c r="E104">
         <v>1</v>
       </c>
-      <c r="F104" s="8">
+      <c r="F104" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16004,7 +16003,7 @@
       <c r="E105">
         <v>1</v>
       </c>
-      <c r="F105" s="8">
+      <c r="F105" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16029,7 +16028,7 @@
       <c r="E106">
         <v>1</v>
       </c>
-      <c r="F106" s="8">
+      <c r="F106" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16054,7 +16053,7 @@
       <c r="E107">
         <v>1</v>
       </c>
-      <c r="F107" s="8">
+      <c r="F107" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16079,7 +16078,7 @@
       <c r="E108">
         <v>1</v>
       </c>
-      <c r="F108" s="8">
+      <c r="F108" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16104,7 +16103,7 @@
       <c r="E109">
         <v>1</v>
       </c>
-      <c r="F109" s="8">
+      <c r="F109" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16129,7 +16128,7 @@
       <c r="E110">
         <v>1</v>
       </c>
-      <c r="F110" s="8">
+      <c r="F110" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16154,7 +16153,7 @@
       <c r="E111">
         <v>1</v>
       </c>
-      <c r="F111" s="8">
+      <c r="F111" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16179,7 +16178,7 @@
       <c r="E112">
         <v>1</v>
       </c>
-      <c r="F112" s="8">
+      <c r="F112" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16204,7 +16203,7 @@
       <c r="E113">
         <v>1</v>
       </c>
-      <c r="F113" s="8">
+      <c r="F113" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16229,7 +16228,7 @@
       <c r="E114">
         <v>1</v>
       </c>
-      <c r="F114" s="8">
+      <c r="F114" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16254,7 +16253,7 @@
       <c r="E115">
         <v>1</v>
       </c>
-      <c r="F115" s="8">
+      <c r="F115" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16279,7 +16278,7 @@
       <c r="E116">
         <v>1</v>
       </c>
-      <c r="F116" s="8">
+      <c r="F116" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16304,7 +16303,7 @@
       <c r="E117">
         <v>1</v>
       </c>
-      <c r="F117" s="8">
+      <c r="F117" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16329,7 +16328,7 @@
       <c r="E118">
         <v>1</v>
       </c>
-      <c r="F118" s="8">
+      <c r="F118" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16354,7 +16353,7 @@
       <c r="E119">
         <v>1</v>
       </c>
-      <c r="F119" s="8">
+      <c r="F119" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16379,7 +16378,7 @@
       <c r="E120">
         <v>1</v>
       </c>
-      <c r="F120" s="8">
+      <c r="F120" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16404,7 +16403,7 @@
       <c r="E121">
         <v>1</v>
       </c>
-      <c r="F121" s="8">
+      <c r="F121" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16429,7 +16428,7 @@
       <c r="E122">
         <v>1</v>
       </c>
-      <c r="F122" s="8">
+      <c r="F122" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16454,7 +16453,7 @@
       <c r="E123">
         <v>1</v>
       </c>
-      <c r="F123" s="8">
+      <c r="F123" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16479,7 +16478,7 @@
       <c r="E124">
         <v>1</v>
       </c>
-      <c r="F124" s="8">
+      <c r="F124" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16504,7 +16503,7 @@
       <c r="E125">
         <v>1</v>
       </c>
-      <c r="F125" s="8">
+      <c r="F125" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16529,7 +16528,7 @@
       <c r="E126">
         <v>1</v>
       </c>
-      <c r="F126" s="8">
+      <c r="F126" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16554,7 +16553,7 @@
       <c r="E127">
         <v>1</v>
       </c>
-      <c r="F127" s="8">
+      <c r="F127" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16579,7 +16578,7 @@
       <c r="E128">
         <v>1</v>
       </c>
-      <c r="F128" s="8">
+      <c r="F128" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16604,7 +16603,7 @@
       <c r="E129">
         <v>1</v>
       </c>
-      <c r="F129" s="8">
+      <c r="F129" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16629,7 +16628,7 @@
       <c r="E130">
         <v>1</v>
       </c>
-      <c r="F130" s="8">
+      <c r="F130" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16654,7 +16653,7 @@
       <c r="E131">
         <v>1</v>
       </c>
-      <c r="F131" s="8">
+      <c r="F131" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16679,7 +16678,7 @@
       <c r="E132">
         <v>1</v>
       </c>
-      <c r="F132" s="8">
+      <c r="F132" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16704,7 +16703,7 @@
       <c r="E133">
         <v>1</v>
       </c>
-      <c r="F133" s="8">
+      <c r="F133" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16729,7 +16728,7 @@
       <c r="E134">
         <v>1</v>
       </c>
-      <c r="F134" s="8">
+      <c r="F134" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16754,7 +16753,7 @@
       <c r="E135">
         <v>1</v>
       </c>
-      <c r="F135" s="8">
+      <c r="F135" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16779,7 +16778,7 @@
       <c r="E136">
         <v>1</v>
       </c>
-      <c r="F136" s="8">
+      <c r="F136" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16804,7 +16803,7 @@
       <c r="E137">
         <v>1</v>
       </c>
-      <c r="F137" s="8">
+      <c r="F137" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16829,7 +16828,7 @@
       <c r="E138">
         <v>1</v>
       </c>
-      <c r="F138" s="8">
+      <c r="F138" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -16854,7 +16853,7 @@
       <c r="E139">
         <v>1</v>
       </c>
-      <c r="F139" s="8">
+      <c r="F139" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16879,7 +16878,7 @@
       <c r="E140">
         <v>1</v>
       </c>
-      <c r="F140" s="8">
+      <c r="F140" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16904,7 +16903,7 @@
       <c r="E141">
         <v>1</v>
       </c>
-      <c r="F141" s="8">
+      <c r="F141" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16929,7 +16928,7 @@
       <c r="E142">
         <v>1</v>
       </c>
-      <c r="F142" s="8">
+      <c r="F142" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16954,7 +16953,7 @@
       <c r="E143">
         <v>1</v>
       </c>
-      <c r="F143" s="8">
+      <c r="F143" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -16979,7 +16978,7 @@
       <c r="E144">
         <v>1</v>
       </c>
-      <c r="F144" s="8">
+      <c r="F144" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17004,7 +17003,7 @@
       <c r="E145">
         <v>1</v>
       </c>
-      <c r="F145" s="8">
+      <c r="F145" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17029,7 +17028,7 @@
       <c r="E146">
         <v>1</v>
       </c>
-      <c r="F146" s="8">
+      <c r="F146" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17054,7 +17053,7 @@
       <c r="E147">
         <v>1</v>
       </c>
-      <c r="F147" s="8">
+      <c r="F147" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17079,7 +17078,7 @@
       <c r="E148">
         <v>1</v>
       </c>
-      <c r="F148" s="8">
+      <c r="F148" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17104,7 +17103,7 @@
       <c r="E149">
         <v>1</v>
       </c>
-      <c r="F149" s="8">
+      <c r="F149" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17129,7 +17128,7 @@
       <c r="E150">
         <v>1</v>
       </c>
-      <c r="F150" s="8">
+      <c r="F150" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17154,7 +17153,7 @@
       <c r="E151">
         <v>1</v>
       </c>
-      <c r="F151" s="8">
+      <c r="F151" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17179,7 +17178,7 @@
       <c r="E152">
         <v>1</v>
       </c>
-      <c r="F152" s="8">
+      <c r="F152" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17204,7 +17203,7 @@
       <c r="E153">
         <v>1</v>
       </c>
-      <c r="F153" s="8">
+      <c r="F153" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17229,7 +17228,7 @@
       <c r="E154">
         <v>1</v>
       </c>
-      <c r="F154" s="8">
+      <c r="F154" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17254,7 +17253,7 @@
       <c r="E155">
         <v>1</v>
       </c>
-      <c r="F155" s="8">
+      <c r="F155" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17279,7 +17278,7 @@
       <c r="E156">
         <v>1</v>
       </c>
-      <c r="F156" s="8">
+      <c r="F156" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17304,7 +17303,7 @@
       <c r="E157">
         <v>1</v>
       </c>
-      <c r="F157" s="8">
+      <c r="F157" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17329,7 +17328,7 @@
       <c r="E158">
         <v>1</v>
       </c>
-      <c r="F158" s="8">
+      <c r="F158" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17354,7 +17353,7 @@
       <c r="E159">
         <v>1</v>
       </c>
-      <c r="F159" s="8">
+      <c r="F159" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17379,7 +17378,7 @@
       <c r="E160">
         <v>1</v>
       </c>
-      <c r="F160" s="8">
+      <c r="F160" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17404,7 +17403,7 @@
       <c r="E161">
         <v>1</v>
       </c>
-      <c r="F161" s="8">
+      <c r="F161" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17429,7 +17428,7 @@
       <c r="E162">
         <v>1</v>
       </c>
-      <c r="F162" s="8">
+      <c r="F162" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17454,7 +17453,7 @@
       <c r="E163">
         <v>1</v>
       </c>
-      <c r="F163" s="8">
+      <c r="F163" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17479,7 +17478,7 @@
       <c r="E164">
         <v>1</v>
       </c>
-      <c r="F164" s="8">
+      <c r="F164" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17504,7 +17503,7 @@
       <c r="E165">
         <v>1</v>
       </c>
-      <c r="F165" s="8">
+      <c r="F165" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17529,7 +17528,7 @@
       <c r="E166">
         <v>1</v>
       </c>
-      <c r="F166" s="8">
+      <c r="F166" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17554,7 +17553,7 @@
       <c r="E167">
         <v>1</v>
       </c>
-      <c r="F167" s="8">
+      <c r="F167" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17579,7 +17578,7 @@
       <c r="E168">
         <v>1</v>
       </c>
-      <c r="F168" s="8">
+      <c r="F168" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17604,7 +17603,7 @@
       <c r="E169">
         <v>1</v>
       </c>
-      <c r="F169" s="8">
+      <c r="F169" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17629,7 +17628,7 @@
       <c r="E170">
         <v>1</v>
       </c>
-      <c r="F170" s="8">
+      <c r="F170" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17654,7 +17653,7 @@
       <c r="E171">
         <v>1</v>
       </c>
-      <c r="F171" s="8">
+      <c r="F171" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17679,7 +17678,7 @@
       <c r="E172">
         <v>1</v>
       </c>
-      <c r="F172" s="8">
+      <c r="F172" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17704,7 +17703,7 @@
       <c r="E173">
         <v>1</v>
       </c>
-      <c r="F173" s="8">
+      <c r="F173" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17729,7 +17728,7 @@
       <c r="E174">
         <v>1</v>
       </c>
-      <c r="F174" s="8">
+      <c r="F174" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17754,7 +17753,7 @@
       <c r="E175">
         <v>1</v>
       </c>
-      <c r="F175" s="8">
+      <c r="F175" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17779,7 +17778,7 @@
       <c r="E176">
         <v>1</v>
       </c>
-      <c r="F176" s="8">
+      <c r="F176" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17804,7 +17803,7 @@
       <c r="E177">
         <v>1</v>
       </c>
-      <c r="F177" s="8">
+      <c r="F177" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -17829,7 +17828,7 @@
       <c r="E178">
         <v>1</v>
       </c>
-      <c r="F178" s="8">
+      <c r="F178" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17854,7 +17853,7 @@
       <c r="E179">
         <v>1</v>
       </c>
-      <c r="F179" s="8">
+      <c r="F179" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17879,7 +17878,7 @@
       <c r="E180">
         <v>1</v>
       </c>
-      <c r="F180" s="8">
+      <c r="F180" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17904,7 +17903,7 @@
       <c r="E181">
         <v>1</v>
       </c>
-      <c r="F181" s="8">
+      <c r="F181" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17929,7 +17928,7 @@
       <c r="E182">
         <v>1</v>
       </c>
-      <c r="F182" s="8">
+      <c r="F182" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17954,7 +17953,7 @@
       <c r="E183">
         <v>1</v>
       </c>
-      <c r="F183" s="8">
+      <c r="F183" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -17979,7 +17978,7 @@
       <c r="E184">
         <v>1</v>
       </c>
-      <c r="F184" s="8">
+      <c r="F184" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18004,7 +18003,7 @@
       <c r="E185">
         <v>1</v>
       </c>
-      <c r="F185" s="8">
+      <c r="F185" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18029,7 +18028,7 @@
       <c r="E186">
         <v>1</v>
       </c>
-      <c r="F186" s="8">
+      <c r="F186" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18054,7 +18053,7 @@
       <c r="E187">
         <v>1</v>
       </c>
-      <c r="F187" s="8">
+      <c r="F187" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18079,7 +18078,7 @@
       <c r="E188">
         <v>1</v>
       </c>
-      <c r="F188" s="8">
+      <c r="F188" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18104,7 +18103,7 @@
       <c r="E189">
         <v>1</v>
       </c>
-      <c r="F189" s="8">
+      <c r="F189" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18129,7 +18128,7 @@
       <c r="E190">
         <v>1</v>
       </c>
-      <c r="F190" s="8">
+      <c r="F190" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18154,7 +18153,7 @@
       <c r="E191">
         <v>1</v>
       </c>
-      <c r="F191" s="8">
+      <c r="F191" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18179,7 +18178,7 @@
       <c r="E192">
         <v>1</v>
       </c>
-      <c r="F192" s="8">
+      <c r="F192" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18204,7 +18203,7 @@
       <c r="E193">
         <v>1</v>
       </c>
-      <c r="F193" s="8">
+      <c r="F193" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18229,7 +18228,7 @@
       <c r="E194">
         <v>1</v>
       </c>
-      <c r="F194" s="8">
+      <c r="F194" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18254,7 +18253,7 @@
       <c r="E195">
         <v>1</v>
       </c>
-      <c r="F195" s="8">
+      <c r="F195" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18279,7 +18278,7 @@
       <c r="E196">
         <v>1</v>
       </c>
-      <c r="F196" s="8">
+      <c r="F196" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18304,7 +18303,7 @@
       <c r="E197">
         <v>1</v>
       </c>
-      <c r="F197" s="8">
+      <c r="F197" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18329,7 +18328,7 @@
       <c r="E198">
         <v>1</v>
       </c>
-      <c r="F198" s="8">
+      <c r="F198" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18354,7 +18353,7 @@
       <c r="E199">
         <v>1</v>
       </c>
-      <c r="F199" s="8">
+      <c r="F199" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18379,7 +18378,7 @@
       <c r="E200">
         <v>1</v>
       </c>
-      <c r="F200" s="8">
+      <c r="F200" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18404,7 +18403,7 @@
       <c r="E201">
         <v>1</v>
       </c>
-      <c r="F201" s="8">
+      <c r="F201" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18429,7 +18428,7 @@
       <c r="E202">
         <v>1</v>
       </c>
-      <c r="F202" s="8">
+      <c r="F202" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18454,7 +18453,7 @@
       <c r="E203">
         <v>1</v>
       </c>
-      <c r="F203" s="8">
+      <c r="F203" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18479,7 +18478,7 @@
       <c r="E204">
         <v>1</v>
       </c>
-      <c r="F204" s="8">
+      <c r="F204" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18504,7 +18503,7 @@
       <c r="E205">
         <v>1</v>
       </c>
-      <c r="F205" s="8">
+      <c r="F205" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18529,7 +18528,7 @@
       <c r="E206">
         <v>1</v>
       </c>
-      <c r="F206" s="8">
+      <c r="F206" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18554,7 +18553,7 @@
       <c r="E207">
         <v>1</v>
       </c>
-      <c r="F207" s="8">
+      <c r="F207" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18579,7 +18578,7 @@
       <c r="E208">
         <v>1</v>
       </c>
-      <c r="F208" s="8">
+      <c r="F208" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -18604,7 +18603,7 @@
       <c r="E209">
         <v>1</v>
       </c>
-      <c r="F209" s="8">
+      <c r="F209" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18629,7 +18628,7 @@
       <c r="E210">
         <v>1</v>
       </c>
-      <c r="F210" s="8">
+      <c r="F210" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18654,7 +18653,7 @@
       <c r="E211">
         <v>1</v>
       </c>
-      <c r="F211" s="8">
+      <c r="F211" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18679,7 +18678,7 @@
       <c r="E212">
         <v>1</v>
       </c>
-      <c r="F212" s="8">
+      <c r="F212" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18704,7 +18703,7 @@
       <c r="E213">
         <v>1</v>
       </c>
-      <c r="F213" s="8">
+      <c r="F213" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18729,7 +18728,7 @@
       <c r="E214">
         <v>1</v>
       </c>
-      <c r="F214" s="8">
+      <c r="F214" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18754,7 +18753,7 @@
       <c r="E215">
         <v>1</v>
       </c>
-      <c r="F215" s="8">
+      <c r="F215" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18779,7 +18778,7 @@
       <c r="E216">
         <v>1</v>
       </c>
-      <c r="F216" s="8">
+      <c r="F216" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18804,7 +18803,7 @@
       <c r="E217">
         <v>1</v>
       </c>
-      <c r="F217" s="8">
+      <c r="F217" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18829,7 +18828,7 @@
       <c r="E218">
         <v>1</v>
       </c>
-      <c r="F218" s="8">
+      <c r="F218" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18854,7 +18853,7 @@
       <c r="E219">
         <v>1</v>
       </c>
-      <c r="F219" s="8">
+      <c r="F219" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18879,7 +18878,7 @@
       <c r="E220">
         <v>1</v>
       </c>
-      <c r="F220" s="8">
+      <c r="F220" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18904,7 +18903,7 @@
       <c r="E221">
         <v>1</v>
       </c>
-      <c r="F221" s="8">
+      <c r="F221" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18929,7 +18928,7 @@
       <c r="E222">
         <v>1</v>
       </c>
-      <c r="F222" s="8">
+      <c r="F222" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18954,7 +18953,7 @@
       <c r="E223">
         <v>1</v>
       </c>
-      <c r="F223" s="8">
+      <c r="F223" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -18979,7 +18978,7 @@
       <c r="E224">
         <v>1</v>
       </c>
-      <c r="F224" s="8">
+      <c r="F224" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19004,7 +19003,7 @@
       <c r="E225">
         <v>1</v>
       </c>
-      <c r="F225" s="8">
+      <c r="F225" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19029,7 +19028,7 @@
       <c r="E226">
         <v>1</v>
       </c>
-      <c r="F226" s="8">
+      <c r="F226" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19054,7 +19053,7 @@
       <c r="E227">
         <v>1</v>
       </c>
-      <c r="F227" s="8">
+      <c r="F227" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19079,7 +19078,7 @@
       <c r="E228">
         <v>1</v>
       </c>
-      <c r="F228" s="8">
+      <c r="F228" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19104,7 +19103,7 @@
       <c r="E229">
         <v>1</v>
       </c>
-      <c r="F229" s="8">
+      <c r="F229" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19129,7 +19128,7 @@
       <c r="E230">
         <v>1</v>
       </c>
-      <c r="F230" s="8">
+      <c r="F230" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19154,7 +19153,7 @@
       <c r="E231">
         <v>1</v>
       </c>
-      <c r="F231" s="8">
+      <c r="F231" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19179,7 +19178,7 @@
       <c r="E232">
         <v>1</v>
       </c>
-      <c r="F232" s="8">
+      <c r="F232" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19204,7 +19203,7 @@
       <c r="E233">
         <v>1</v>
       </c>
-      <c r="F233" s="8">
+      <c r="F233" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19229,7 +19228,7 @@
       <c r="E234">
         <v>1</v>
       </c>
-      <c r="F234" s="8">
+      <c r="F234" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19254,7 +19253,7 @@
       <c r="E235">
         <v>1</v>
       </c>
-      <c r="F235" s="8">
+      <c r="F235" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19279,7 +19278,7 @@
       <c r="E236">
         <v>1</v>
       </c>
-      <c r="F236" s="8">
+      <c r="F236" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19304,7 +19303,7 @@
       <c r="E237">
         <v>1</v>
       </c>
-      <c r="F237" s="8">
+      <c r="F237" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19329,7 +19328,7 @@
       <c r="E238">
         <v>1</v>
       </c>
-      <c r="F238" s="8">
+      <c r="F238" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19354,7 +19353,7 @@
       <c r="E239">
         <v>1</v>
       </c>
-      <c r="F239" s="8">
+      <c r="F239" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19379,7 +19378,7 @@
       <c r="E240">
         <v>1</v>
       </c>
-      <c r="F240" s="8">
+      <c r="F240" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19404,7 +19403,7 @@
       <c r="E241">
         <v>1</v>
       </c>
-      <c r="F241" s="8">
+      <c r="F241" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19429,7 +19428,7 @@
       <c r="E242">
         <v>1</v>
       </c>
-      <c r="F242" s="8">
+      <c r="F242" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19454,7 +19453,7 @@
       <c r="E243">
         <v>1</v>
       </c>
-      <c r="F243" s="8">
+      <c r="F243" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19479,7 +19478,7 @@
       <c r="E244">
         <v>1</v>
       </c>
-      <c r="F244" s="8">
+      <c r="F244" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19504,7 +19503,7 @@
       <c r="E245">
         <v>1</v>
       </c>
-      <c r="F245" s="8">
+      <c r="F245" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19529,7 +19528,7 @@
       <c r="E246">
         <v>1</v>
       </c>
-      <c r="F246" s="8">
+      <c r="F246" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19554,7 +19553,7 @@
       <c r="E247">
         <v>1</v>
       </c>
-      <c r="F247" s="8">
+      <c r="F247" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19579,7 +19578,7 @@
       <c r="E248">
         <v>1</v>
       </c>
-      <c r="F248" s="8">
+      <c r="F248" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19604,7 +19603,7 @@
       <c r="E249">
         <v>1</v>
       </c>
-      <c r="F249" s="8">
+      <c r="F249" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19629,7 +19628,7 @@
       <c r="E250">
         <v>1</v>
       </c>
-      <c r="F250" s="8">
+      <c r="F250" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19654,7 +19653,7 @@
       <c r="E251">
         <v>1</v>
       </c>
-      <c r="F251" s="8">
+      <c r="F251" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19679,7 +19678,7 @@
       <c r="E252">
         <v>1</v>
       </c>
-      <c r="F252" s="8">
+      <c r="F252" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19704,7 +19703,7 @@
       <c r="E253">
         <v>1</v>
       </c>
-      <c r="F253" s="8">
+      <c r="F253" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19729,7 +19728,7 @@
       <c r="E254">
         <v>1</v>
       </c>
-      <c r="F254" s="8">
+      <c r="F254" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19754,7 +19753,7 @@
       <c r="E255">
         <v>1</v>
       </c>
-      <c r="F255" s="8">
+      <c r="F255" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19779,7 +19778,7 @@
       <c r="E256">
         <v>1</v>
       </c>
-      <c r="F256" s="8">
+      <c r="F256" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19804,7 +19803,7 @@
       <c r="E257">
         <v>1</v>
       </c>
-      <c r="F257" s="8">
+      <c r="F257" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19829,7 +19828,7 @@
       <c r="E258">
         <v>1</v>
       </c>
-      <c r="F258" s="8">
+      <c r="F258" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19854,7 +19853,7 @@
       <c r="E259">
         <v>1</v>
       </c>
-      <c r="F259" s="8">
+      <c r="F259" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19879,7 +19878,7 @@
       <c r="E260">
         <v>1</v>
       </c>
-      <c r="F260" s="8">
+      <c r="F260" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19904,7 +19903,7 @@
       <c r="E261">
         <v>1</v>
       </c>
-      <c r="F261" s="8">
+      <c r="F261" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -19929,7 +19928,7 @@
       <c r="E262">
         <v>1</v>
       </c>
-      <c r="F262" s="8">
+      <c r="F262" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19954,7 +19953,7 @@
       <c r="E263">
         <v>1</v>
       </c>
-      <c r="F263" s="8">
+      <c r="F263" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -19979,7 +19978,7 @@
       <c r="E264">
         <v>1</v>
       </c>
-      <c r="F264" s="8">
+      <c r="F264" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20004,7 +20003,7 @@
       <c r="E265">
         <v>1</v>
       </c>
-      <c r="F265" s="8">
+      <c r="F265" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20029,7 +20028,7 @@
       <c r="E266">
         <v>1</v>
       </c>
-      <c r="F266" s="8">
+      <c r="F266" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20054,7 +20053,7 @@
       <c r="E267">
         <v>1</v>
       </c>
-      <c r="F267" s="8">
+      <c r="F267" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20079,7 +20078,7 @@
       <c r="E268">
         <v>1</v>
       </c>
-      <c r="F268" s="8">
+      <c r="F268" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20104,7 +20103,7 @@
       <c r="E269">
         <v>1</v>
       </c>
-      <c r="F269" s="8">
+      <c r="F269" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20129,7 +20128,7 @@
       <c r="E270">
         <v>1</v>
       </c>
-      <c r="F270" s="8">
+      <c r="F270" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20154,7 +20153,7 @@
       <c r="E271">
         <v>1</v>
       </c>
-      <c r="F271" s="8">
+      <c r="F271" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20179,7 +20178,7 @@
       <c r="E272">
         <v>1</v>
       </c>
-      <c r="F272" s="8">
+      <c r="F272" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20204,7 +20203,7 @@
       <c r="E273">
         <v>1</v>
       </c>
-      <c r="F273" s="8">
+      <c r="F273" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20229,7 +20228,7 @@
       <c r="E274">
         <v>1</v>
       </c>
-      <c r="F274" s="8">
+      <c r="F274" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20254,7 +20253,7 @@
       <c r="E275">
         <v>1</v>
       </c>
-      <c r="F275" s="8">
+      <c r="F275" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20279,7 +20278,7 @@
       <c r="E276">
         <v>1</v>
       </c>
-      <c r="F276" s="8">
+      <c r="F276" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20304,7 +20303,7 @@
       <c r="E277">
         <v>1</v>
       </c>
-      <c r="F277" s="8">
+      <c r="F277" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20329,7 +20328,7 @@
       <c r="E278">
         <v>1</v>
       </c>
-      <c r="F278" s="8">
+      <c r="F278" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20354,7 +20353,7 @@
       <c r="E279">
         <v>1</v>
       </c>
-      <c r="F279" s="8">
+      <c r="F279" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20379,7 +20378,7 @@
       <c r="E280">
         <v>1</v>
       </c>
-      <c r="F280" s="8">
+      <c r="F280" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20404,7 +20403,7 @@
       <c r="E281">
         <v>1</v>
       </c>
-      <c r="F281" s="8">
+      <c r="F281" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20429,7 +20428,7 @@
       <c r="E282">
         <v>1</v>
       </c>
-      <c r="F282" s="8">
+      <c r="F282" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20454,7 +20453,7 @@
       <c r="E283">
         <v>1</v>
       </c>
-      <c r="F283" s="8">
+      <c r="F283" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20479,7 +20478,7 @@
       <c r="E284">
         <v>1</v>
       </c>
-      <c r="F284" s="8">
+      <c r="F284" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20504,7 +20503,7 @@
       <c r="E285">
         <v>1</v>
       </c>
-      <c r="F285" s="8">
+      <c r="F285" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20529,7 +20528,7 @@
       <c r="E286">
         <v>1</v>
       </c>
-      <c r="F286" s="8">
+      <c r="F286" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20554,7 +20553,7 @@
       <c r="E287">
         <v>1</v>
       </c>
-      <c r="F287" s="8">
+      <c r="F287" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20579,7 +20578,7 @@
       <c r="E288">
         <v>1</v>
       </c>
-      <c r="F288" s="8">
+      <c r="F288" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20604,7 +20603,7 @@
       <c r="E289">
         <v>1</v>
       </c>
-      <c r="F289" s="8">
+      <c r="F289" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20629,7 +20628,7 @@
       <c r="E290">
         <v>1</v>
       </c>
-      <c r="F290" s="8">
+      <c r="F290" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20654,7 +20653,7 @@
       <c r="E291">
         <v>1</v>
       </c>
-      <c r="F291" s="8">
+      <c r="F291" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20679,7 +20678,7 @@
       <c r="E292">
         <v>1</v>
       </c>
-      <c r="F292" s="8">
+      <c r="F292" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20704,7 +20703,7 @@
       <c r="E293">
         <v>1</v>
       </c>
-      <c r="F293" s="8">
+      <c r="F293" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20729,7 +20728,7 @@
       <c r="E294">
         <v>1</v>
       </c>
-      <c r="F294" s="8">
+      <c r="F294" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20754,7 +20753,7 @@
       <c r="E295">
         <v>1</v>
       </c>
-      <c r="F295" s="8">
+      <c r="F295" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20779,7 +20778,7 @@
       <c r="E296">
         <v>1</v>
       </c>
-      <c r="F296" s="8">
+      <c r="F296" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20804,7 +20803,7 @@
       <c r="E297">
         <v>1</v>
       </c>
-      <c r="F297" s="8">
+      <c r="F297" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20829,7 +20828,7 @@
       <c r="E298">
         <v>1</v>
       </c>
-      <c r="F298" s="8">
+      <c r="F298" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20854,7 +20853,7 @@
       <c r="E299">
         <v>1</v>
       </c>
-      <c r="F299" s="8">
+      <c r="F299" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20879,7 +20878,7 @@
       <c r="E300">
         <v>1</v>
       </c>
-      <c r="F300" s="8">
+      <c r="F300" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20904,7 +20903,7 @@
       <c r="E301">
         <v>1</v>
       </c>
-      <c r="F301" s="8">
+      <c r="F301" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20929,7 +20928,7 @@
       <c r="E302">
         <v>1</v>
       </c>
-      <c r="F302" s="8">
+      <c r="F302" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -20954,7 +20953,7 @@
       <c r="E303">
         <v>1</v>
       </c>
-      <c r="F303" s="8">
+      <c r="F303" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -20979,7 +20978,7 @@
       <c r="E304">
         <v>1</v>
       </c>
-      <c r="F304" s="8">
+      <c r="F304" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -21004,7 +21003,7 @@
       <c r="E305">
         <v>1</v>
       </c>
-      <c r="F305" s="8">
+      <c r="F305" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21029,7 +21028,7 @@
       <c r="E306">
         <v>1</v>
       </c>
-      <c r="F306" s="8">
+      <c r="F306" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21054,7 +21053,7 @@
       <c r="E307">
         <v>1</v>
       </c>
-      <c r="F307" s="8">
+      <c r="F307" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -21079,7 +21078,7 @@
       <c r="E308">
         <v>1</v>
       </c>
-      <c r="F308" s="8">
+      <c r="F308" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -21104,7 +21103,7 @@
       <c r="E309">
         <v>1</v>
       </c>
-      <c r="F309" s="8">
+      <c r="F309" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21129,7 +21128,7 @@
       <c r="E310">
         <v>1</v>
       </c>
-      <c r="F310" s="8">
+      <c r="F310" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>1</v>
       </c>
@@ -21154,7 +21153,7 @@
       <c r="E311">
         <v>0</v>
       </c>
-      <c r="F311" s="8">
+      <c r="F311" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21179,7 +21178,7 @@
       <c r="E312">
         <v>0</v>
       </c>
-      <c r="F312" s="8">
+      <c r="F312" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21204,7 +21203,7 @@
       <c r="E313">
         <v>0</v>
       </c>
-      <c r="F313" s="8">
+      <c r="F313" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21229,7 +21228,7 @@
       <c r="E314">
         <v>0</v>
       </c>
-      <c r="F314" s="8">
+      <c r="F314" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21254,7 +21253,7 @@
       <c r="E315">
         <v>0</v>
       </c>
-      <c r="F315" s="8">
+      <c r="F315" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21279,7 +21278,7 @@
       <c r="E316">
         <v>0</v>
       </c>
-      <c r="F316" s="8">
+      <c r="F316" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21304,7 +21303,7 @@
       <c r="E317">
         <v>0</v>
       </c>
-      <c r="F317" s="8">
+      <c r="F317" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21329,7 +21328,7 @@
       <c r="E318">
         <v>0</v>
       </c>
-      <c r="F318" s="8">
+      <c r="F318" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21354,7 +21353,7 @@
       <c r="E319">
         <v>0</v>
       </c>
-      <c r="F319" s="8">
+      <c r="F319" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21379,7 +21378,7 @@
       <c r="E320">
         <v>0</v>
       </c>
-      <c r="F320" s="8">
+      <c r="F320" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21404,7 +21403,7 @@
       <c r="E321">
         <v>0</v>
       </c>
-      <c r="F321" s="8">
+      <c r="F321" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21429,7 +21428,7 @@
       <c r="E322">
         <v>0</v>
       </c>
-      <c r="F322" s="8">
+      <c r="F322" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21454,7 +21453,7 @@
       <c r="E323">
         <v>0</v>
       </c>
-      <c r="F323" s="8">
+      <c r="F323" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21479,7 +21478,7 @@
       <c r="E324">
         <v>0</v>
       </c>
-      <c r="F324" s="8">
+      <c r="F324" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21504,7 +21503,7 @@
       <c r="E325">
         <v>0</v>
       </c>
-      <c r="F325" s="8">
+      <c r="F325" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21529,7 +21528,7 @@
       <c r="E326">
         <v>0</v>
       </c>
-      <c r="F326" s="8">
+      <c r="F326" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21554,7 +21553,7 @@
       <c r="E327">
         <v>0</v>
       </c>
-      <c r="F327" s="8">
+      <c r="F327" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21579,7 +21578,7 @@
       <c r="E328">
         <v>0</v>
       </c>
-      <c r="F328" s="8">
+      <c r="F328" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21604,7 +21603,7 @@
       <c r="E329">
         <v>0</v>
       </c>
-      <c r="F329" s="8">
+      <c r="F329" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21629,7 +21628,7 @@
       <c r="E330">
         <v>0</v>
       </c>
-      <c r="F330" s="8">
+      <c r="F330" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21654,7 +21653,7 @@
       <c r="E331">
         <v>0</v>
       </c>
-      <c r="F331" s="8">
+      <c r="F331" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21679,7 +21678,7 @@
       <c r="E332">
         <v>0</v>
       </c>
-      <c r="F332" s="8">
+      <c r="F332" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21704,7 +21703,7 @@
       <c r="E333">
         <v>0</v>
       </c>
-      <c r="F333" s="8">
+      <c r="F333" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21729,7 +21728,7 @@
       <c r="E334">
         <v>0</v>
       </c>
-      <c r="F334" s="8">
+      <c r="F334" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21754,7 +21753,7 @@
       <c r="E335">
         <v>0</v>
       </c>
-      <c r="F335" s="8">
+      <c r="F335" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21779,7 +21778,7 @@
       <c r="E336">
         <v>0</v>
       </c>
-      <c r="F336" s="8">
+      <c r="F336" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21804,7 +21803,7 @@
       <c r="E337">
         <v>0</v>
       </c>
-      <c r="F337" s="8">
+      <c r="F337" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21829,7 +21828,7 @@
       <c r="E338">
         <v>0</v>
       </c>
-      <c r="F338" s="8">
+      <c r="F338" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21854,7 +21853,7 @@
       <c r="E339">
         <v>0</v>
       </c>
-      <c r="F339" s="8">
+      <c r="F339" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21879,7 +21878,7 @@
       <c r="E340">
         <v>0</v>
       </c>
-      <c r="F340" s="8">
+      <c r="F340" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21904,7 +21903,7 @@
       <c r="E341">
         <v>0</v>
       </c>
-      <c r="F341" s="8">
+      <c r="F341" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21929,7 +21928,7 @@
       <c r="E342">
         <v>0</v>
       </c>
-      <c r="F342" s="8">
+      <c r="F342" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21954,7 +21953,7 @@
       <c r="E343">
         <v>0</v>
       </c>
-      <c r="F343" s="8">
+      <c r="F343" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -21979,7 +21978,7 @@
       <c r="E344">
         <v>0</v>
       </c>
-      <c r="F344" s="8">
+      <c r="F344" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22004,7 +22003,7 @@
       <c r="E345">
         <v>0</v>
       </c>
-      <c r="F345" s="8">
+      <c r="F345" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22029,7 +22028,7 @@
       <c r="E346">
         <v>0</v>
       </c>
-      <c r="F346" s="8">
+      <c r="F346" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22054,7 +22053,7 @@
       <c r="E347">
         <v>0</v>
       </c>
-      <c r="F347" s="8">
+      <c r="F347" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22079,7 +22078,7 @@
       <c r="E348">
         <v>0</v>
       </c>
-      <c r="F348" s="8">
+      <c r="F348" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22104,7 +22103,7 @@
       <c r="E349">
         <v>0</v>
       </c>
-      <c r="F349" s="8">
+      <c r="F349" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22129,7 +22128,7 @@
       <c r="E350">
         <v>0</v>
       </c>
-      <c r="F350" s="8">
+      <c r="F350" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22154,7 +22153,7 @@
       <c r="E351">
         <v>0</v>
       </c>
-      <c r="F351" s="8">
+      <c r="F351" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22179,7 +22178,7 @@
       <c r="E352">
         <v>0</v>
       </c>
-      <c r="F352" s="8">
+      <c r="F352" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22204,7 +22203,7 @@
       <c r="E353">
         <v>0</v>
       </c>
-      <c r="F353" s="8">
+      <c r="F353" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22229,7 +22228,7 @@
       <c r="E354">
         <v>0</v>
       </c>
-      <c r="F354" s="8">
+      <c r="F354" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22254,7 +22253,7 @@
       <c r="E355">
         <v>0</v>
       </c>
-      <c r="F355" s="8">
+      <c r="F355" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22279,7 +22278,7 @@
       <c r="E356">
         <v>0</v>
       </c>
-      <c r="F356" s="8">
+      <c r="F356" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22304,7 +22303,7 @@
       <c r="E357">
         <v>0</v>
       </c>
-      <c r="F357" s="8">
+      <c r="F357" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22329,7 +22328,7 @@
       <c r="E358">
         <v>0</v>
       </c>
-      <c r="F358" s="8">
+      <c r="F358" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22354,7 +22353,7 @@
       <c r="E359">
         <v>0</v>
       </c>
-      <c r="F359" s="8">
+      <c r="F359" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22379,7 +22378,7 @@
       <c r="E360">
         <v>0</v>
       </c>
-      <c r="F360" s="8">
+      <c r="F360" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22404,7 +22403,7 @@
       <c r="E361">
         <v>0</v>
       </c>
-      <c r="F361" s="8">
+      <c r="F361" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22429,7 +22428,7 @@
       <c r="E362">
         <v>0</v>
       </c>
-      <c r="F362" s="8">
+      <c r="F362" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22454,7 +22453,7 @@
       <c r="E363">
         <v>0</v>
       </c>
-      <c r="F363" s="8">
+      <c r="F363" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22479,7 +22478,7 @@
       <c r="E364">
         <v>0</v>
       </c>
-      <c r="F364" s="8">
+      <c r="F364" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22504,7 +22503,7 @@
       <c r="E365">
         <v>0</v>
       </c>
-      <c r="F365" s="8">
+      <c r="F365" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22529,7 +22528,7 @@
       <c r="E366">
         <v>0</v>
       </c>
-      <c r="F366" s="8">
+      <c r="F366" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22554,7 +22553,7 @@
       <c r="E367">
         <v>0</v>
       </c>
-      <c r="F367" s="8">
+      <c r="F367" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22579,7 +22578,7 @@
       <c r="E368">
         <v>0</v>
       </c>
-      <c r="F368" s="8">
+      <c r="F368" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22604,7 +22603,7 @@
       <c r="E369">
         <v>0</v>
       </c>
-      <c r="F369" s="8">
+      <c r="F369" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22629,7 +22628,7 @@
       <c r="E370">
         <v>0</v>
       </c>
-      <c r="F370" s="8">
+      <c r="F370" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22654,7 +22653,7 @@
       <c r="E371">
         <v>0</v>
       </c>
-      <c r="F371" s="8">
+      <c r="F371" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22679,7 +22678,7 @@
       <c r="E372">
         <v>0</v>
       </c>
-      <c r="F372" s="8">
+      <c r="F372" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22704,7 +22703,7 @@
       <c r="E373">
         <v>0</v>
       </c>
-      <c r="F373" s="8">
+      <c r="F373" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22729,7 +22728,7 @@
       <c r="E374">
         <v>0</v>
       </c>
-      <c r="F374" s="8">
+      <c r="F374" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22754,7 +22753,7 @@
       <c r="E375">
         <v>0</v>
       </c>
-      <c r="F375" s="8">
+      <c r="F375" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22779,7 +22778,7 @@
       <c r="E376">
         <v>0</v>
       </c>
-      <c r="F376" s="8">
+      <c r="F376" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22804,7 +22803,7 @@
       <c r="E377">
         <v>0</v>
       </c>
-      <c r="F377" s="8">
+      <c r="F377" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22829,7 +22828,7 @@
       <c r="E378">
         <v>0</v>
       </c>
-      <c r="F378" s="8">
+      <c r="F378" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22854,7 +22853,7 @@
       <c r="E379">
         <v>0</v>
       </c>
-      <c r="F379" s="8">
+      <c r="F379" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22879,7 +22878,7 @@
       <c r="E380">
         <v>0</v>
       </c>
-      <c r="F380" s="8">
+      <c r="F380" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22904,7 +22903,7 @@
       <c r="E381">
         <v>0</v>
       </c>
-      <c r="F381" s="8">
+      <c r="F381" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22929,7 +22928,7 @@
       <c r="E382">
         <v>0</v>
       </c>
-      <c r="F382" s="8">
+      <c r="F382" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22954,7 +22953,7 @@
       <c r="E383">
         <v>0</v>
       </c>
-      <c r="F383" s="8">
+      <c r="F383" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -22979,7 +22978,7 @@
       <c r="E384">
         <v>0</v>
       </c>
-      <c r="F384" s="8">
+      <c r="F384" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23004,7 +23003,7 @@
       <c r="E385">
         <v>0</v>
       </c>
-      <c r="F385" s="8">
+      <c r="F385" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23029,7 +23028,7 @@
       <c r="E386">
         <v>0</v>
       </c>
-      <c r="F386" s="8">
+      <c r="F386" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23054,7 +23053,7 @@
       <c r="E387">
         <v>0</v>
       </c>
-      <c r="F387" s="8">
+      <c r="F387" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23079,7 +23078,7 @@
       <c r="E388">
         <v>0</v>
       </c>
-      <c r="F388" s="8">
+      <c r="F388" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23104,7 +23103,7 @@
       <c r="E389">
         <v>0</v>
       </c>
-      <c r="F389" s="8">
+      <c r="F389" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23129,7 +23128,7 @@
       <c r="E390">
         <v>0</v>
       </c>
-      <c r="F390" s="8">
+      <c r="F390" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23154,7 +23153,7 @@
       <c r="E391">
         <v>0</v>
       </c>
-      <c r="F391" s="8">
+      <c r="F391" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23179,7 +23178,7 @@
       <c r="E392">
         <v>0</v>
       </c>
-      <c r="F392" s="8">
+      <c r="F392" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23204,7 +23203,7 @@
       <c r="E393">
         <v>0</v>
       </c>
-      <c r="F393" s="8">
+      <c r="F393" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23229,7 +23228,7 @@
       <c r="E394">
         <v>0</v>
       </c>
-      <c r="F394" s="8">
+      <c r="F394" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23254,7 +23253,7 @@
       <c r="E395">
         <v>0</v>
       </c>
-      <c r="F395" s="8">
+      <c r="F395" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23279,7 +23278,7 @@
       <c r="E396">
         <v>0</v>
       </c>
-      <c r="F396" s="8">
+      <c r="F396" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23304,7 +23303,7 @@
       <c r="E397">
         <v>0</v>
       </c>
-      <c r="F397" s="8">
+      <c r="F397" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23329,7 +23328,7 @@
       <c r="E398">
         <v>0</v>
       </c>
-      <c r="F398" s="8">
+      <c r="F398" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23354,7 +23353,7 @@
       <c r="E399">
         <v>0</v>
       </c>
-      <c r="F399" s="8">
+      <c r="F399" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23379,7 +23378,7 @@
       <c r="E400">
         <v>0</v>
       </c>
-      <c r="F400" s="8">
+      <c r="F400" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -23404,7 +23403,7 @@
       <c r="E401">
         <v>0</v>
       </c>
-      <c r="F401" s="8">
+      <c r="F401" s="7">
         <f>IF(AND(Table1[[#This Row],[Predicted Outcome]]=1,Table1[[#This Row],[Actual Outcome]]=1),1,0)</f>
         <v>0</v>
       </c>
@@ -24325,17 +24324,17 @@
       <c r="A4" s="4">
         <v>0</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4">
         <v>40</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4">
         <v>9</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>0.17496599286467901</v>
       </c>
       <c r="G4">
-        <f>B4-C4</f>
+        <f t="shared" ref="G4:G13" si="0">B4-C4</f>
         <v>31</v>
       </c>
       <c r="H4">
@@ -24343,7 +24342,7 @@
         <v>9</v>
       </c>
       <c r="I4" s="2">
-        <f>(H4)/$H$13</f>
+        <f t="shared" ref="I4:I13" si="1">(H4)/$H$13</f>
         <v>3.4883720930232558E-2</v>
       </c>
       <c r="J4">
@@ -24351,10 +24350,10 @@
         <v>31</v>
       </c>
       <c r="K4" s="2">
-        <f>(J4)/$J$13</f>
+        <f t="shared" ref="K4:K13" si="2">(J4)/$J$13</f>
         <v>0.21830985915492956</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>3400</v>
       </c>
@@ -24363,17 +24362,17 @@
       <c r="A5" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5">
         <v>40</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5">
         <v>5</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="11">
         <v>0.35881366224141897</v>
       </c>
       <c r="G5">
-        <f>B5-C5</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="H5">
@@ -24381,18 +24380,18 @@
         <v>14</v>
       </c>
       <c r="I5" s="2">
-        <f>(H5)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>5.4263565891472867E-2</v>
       </c>
       <c r="J5">
         <f>SUM($G$4:G5)</f>
         <v>66</v>
       </c>
-      <c r="K5" s="6">
-        <f>(J5)/$J$13</f>
+      <c r="K5" s="5">
+        <f t="shared" si="2"/>
         <v>0.46478873239436619</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>12400</v>
       </c>
@@ -24401,17 +24400,17 @@
       <c r="A6" s="4">
         <v>2</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6">
         <v>40</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6">
         <v>23</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>0.47584258697556497</v>
       </c>
       <c r="G6">
-        <f>B6-C6</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="H6">
@@ -24419,18 +24418,18 @@
         <v>37</v>
       </c>
       <c r="I6" s="2">
-        <f>(H6)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.1434108527131783</v>
       </c>
       <c r="J6">
         <f>SUM($G$4:G6)</f>
         <v>83</v>
       </c>
-      <c r="K6" s="6">
-        <f>(J6)/$J$13</f>
+      <c r="K6" s="5">
+        <f t="shared" si="2"/>
         <v>0.58450704225352113</v>
       </c>
-      <c r="L6" s="10">
+      <c r="L6" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-3800</v>
       </c>
@@ -24439,17 +24438,17 @@
       <c r="A7" s="4">
         <v>3</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7">
         <v>40</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7">
         <v>30</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <v>0.56482777819684904</v>
       </c>
       <c r="G7">
-        <f>B7-C7</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="H7">
@@ -24457,18 +24456,18 @@
         <v>67</v>
       </c>
       <c r="I7" s="2">
-        <f>(H7)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.25968992248062017</v>
       </c>
       <c r="J7">
         <f>SUM($G$4:G7)</f>
         <v>93</v>
       </c>
-      <c r="K7" s="6">
-        <f>(J7)/$J$13</f>
+      <c r="K7" s="5">
+        <f t="shared" si="2"/>
         <v>0.65492957746478875</v>
       </c>
-      <c r="L7" s="10">
+      <c r="L7" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-29800</v>
       </c>
@@ -24477,17 +24476,17 @@
       <c r="A8" s="4">
         <v>4</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8">
         <v>40</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8">
         <v>33</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <v>0.63757566072097405</v>
       </c>
       <c r="G8">
-        <f>B8-C8</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="H8">
@@ -24495,18 +24494,18 @@
         <v>100</v>
       </c>
       <c r="I8" s="2">
-        <f>(H8)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.38759689922480622</v>
       </c>
       <c r="J8">
         <f>SUM($G$4:G8)</f>
         <v>100</v>
       </c>
-      <c r="K8" s="6">
-        <f>(J8)/$J$13</f>
+      <c r="K8" s="5">
+        <f t="shared" si="2"/>
         <v>0.70422535211267601</v>
       </c>
-      <c r="L8" s="10">
+      <c r="L8" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-60000</v>
       </c>
@@ -24515,17 +24514,17 @@
       <c r="A9" s="4">
         <v>5</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9">
         <v>40</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9">
         <v>32</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <v>0.68823276453429405</v>
       </c>
       <c r="G9">
-        <f>B9-C9</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="H9">
@@ -24533,18 +24532,18 @@
         <v>132</v>
       </c>
       <c r="I9" s="2">
-        <f>(H9)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.51162790697674421</v>
       </c>
       <c r="J9">
         <f>SUM($G$4:G9)</f>
         <v>108</v>
       </c>
-      <c r="K9" s="6">
-        <f>(J9)/$J$13</f>
+      <c r="K9" s="5">
+        <f t="shared" si="2"/>
         <v>0.76056338028169013</v>
       </c>
-      <c r="L9" s="10">
+      <c r="L9" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-88800</v>
       </c>
@@ -24553,17 +24552,17 @@
       <c r="A10" s="4">
         <v>6</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10">
         <v>40</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10">
         <v>31</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <v>0.73607145012303798</v>
       </c>
       <c r="G10">
-        <f>B10-C10</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="H10">
@@ -24571,18 +24570,18 @@
         <v>163</v>
       </c>
       <c r="I10" s="2">
-        <f>(H10)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.63178294573643412</v>
       </c>
       <c r="J10">
         <f>SUM($G$4:G10)</f>
         <v>117</v>
       </c>
-      <c r="K10" s="6">
-        <f>(J10)/$J$13</f>
+      <c r="K10" s="5">
+        <f t="shared" si="2"/>
         <v>0.823943661971831</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-116200</v>
       </c>
@@ -24591,17 +24590,17 @@
       <c r="A11" s="4">
         <v>7</v>
       </c>
-      <c r="B11" s="5">
+      <c r="B11">
         <v>40</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11">
         <v>33</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="5">
         <v>0.790000147675743</v>
       </c>
       <c r="G11">
-        <f>B11-C11</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="H11">
@@ -24609,18 +24608,18 @@
         <v>196</v>
       </c>
       <c r="I11" s="2">
-        <f>(H11)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.75968992248062017</v>
       </c>
       <c r="J11">
         <f>SUM($G$4:G11)</f>
         <v>124</v>
       </c>
-      <c r="K11" s="6">
-        <f>(J11)/$J$13</f>
+      <c r="K11" s="5">
+        <f t="shared" si="2"/>
         <v>0.87323943661971826</v>
       </c>
-      <c r="L11" s="10">
+      <c r="L11" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-146400</v>
       </c>
@@ -24629,17 +24628,17 @@
       <c r="A12" s="4">
         <v>8</v>
       </c>
-      <c r="B12" s="5">
+      <c r="B12">
         <v>40</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12">
         <v>31</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="5">
         <v>0.84607193303260098</v>
       </c>
       <c r="G12">
-        <f>B12-C12</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="H12">
@@ -24647,18 +24646,18 @@
         <v>227</v>
       </c>
       <c r="I12" s="2">
-        <f>(H12)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>0.87984496124031009</v>
       </c>
       <c r="J12">
         <f>SUM($G$4:G12)</f>
         <v>133</v>
       </c>
-      <c r="K12" s="6">
-        <f>(J12)/$J$13</f>
+      <c r="K12" s="5">
+        <f t="shared" si="2"/>
         <v>0.93661971830985913</v>
       </c>
-      <c r="L12" s="10">
+      <c r="L12" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-173800</v>
       </c>
@@ -24667,17 +24666,17 @@
       <c r="A13" s="4">
         <v>9</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13">
         <v>40</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13">
         <v>31</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <v>0.88753490911426602</v>
       </c>
       <c r="G13">
-        <f>B13-C13</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="H13">
@@ -24685,18 +24684,18 @@
         <v>258</v>
       </c>
       <c r="I13" s="2">
-        <f>(H13)/$H$13</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="J13">
         <f>SUM($G$4:G13)</f>
         <v>142</v>
       </c>
-      <c r="K13" s="6">
-        <f>(J13)/$J$13</f>
-        <v>1</v>
-      </c>
-      <c r="L13" s="10">
+      <c r="K13" s="5">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="L13" s="8">
         <f>Table3[[#This Row],[Cumulative Safe Loans]]*$I$18-Table3[[#This Row],[Cumulative Defaults]]*$I$17</f>
         <v>-201200</v>
       </c>
@@ -24705,52 +24704,52 @@
       <c r="A14" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14">
         <v>400</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14">
         <v>258</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <v>0.17496599286467901</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="K16" s="15" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="K16" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="L16" s="17">
+      <c r="L16" s="14">
         <f>L5</f>
         <v>12400</v>
       </c>
     </row>
     <row r="17" spans="7:12" x14ac:dyDescent="0.2">
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="H17" s="12"/>
-      <c r="I17" s="13">
+      <c r="H17" s="17"/>
+      <c r="I17" s="10">
         <v>1000</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="K17" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="L17" s="16">
+      <c r="L17" s="13">
         <f>D5</f>
         <v>0.35881366224141897</v>
       </c>
     </row>
     <row r="18" spans="7:12" x14ac:dyDescent="0.2">
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="H18" s="12"/>
-      <c r="I18" s="13">
+      <c r="H18" s="17"/>
+      <c r="I18" s="10">
         <v>400</v>
       </c>
     </row>

</xml_diff>